<commit_message>
Update analysis notebooks and model results
</commit_message>
<xml_diff>
--- a/model_analysis/generic_kl_multiple_single_variable_analysis.xlsx
+++ b/model_analysis/generic_kl_multiple_single_variable_analysis.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="18400" activeTab="1"/>
+    <workbookView windowWidth="17830" firstSheet="4" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -17,6 +17,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Calculated Yield Strength_max_c'!$B$1:$B$371</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Interant d electrons_max_change'!$B$1:$B$371</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -1182,7 +1183,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1193,13 +1194,6 @@
     <font>
       <b/>
       <sz val="11"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -1667,28 +1661,31 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1697,118 +1694,115 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -2164,7 +2158,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
@@ -2175,10 +2169,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:C371"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="2"/>
   <cols>
-    <col min="2" max="2" width="50.8181818181818" customWidth="1"/>
-    <col min="3" max="3" width="12.8181818181818"/>
+    <col min="2" max="2" width="50.8166666666667" customWidth="1"/>
+    <col min="3" max="3" width="12.8166666666667"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -6263,7 +6257,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B1:B371">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="B1:B371" etc:filterBottomFollowUsedRange="0">
     <extLst/>
   </autoFilter>
   <sortState ref="A2:C371">
@@ -6278,7 +6272,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:C371"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="2"/>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
@@ -10371,7 +10365,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:C371"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="2"/>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
@@ -14464,7 +14458,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:C371"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="2"/>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
@@ -18557,7 +18551,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:C371"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="2"/>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
@@ -22648,9 +22642,14 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:C371"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="2"/>
+  <cols>
+    <col min="1" max="1" width="71.5" customWidth="1"/>
+    <col min="2" max="2" width="45.375" customWidth="1"/>
+    <col min="3" max="3" width="32.875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
@@ -22663,7 +22662,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" hidden="1" spans="1:3">
       <c r="A2" t="s">
         <v>356</v>
       </c>
@@ -22674,7 +22673,7 @@
         <v>381.909496512858</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" hidden="1" spans="1:3">
       <c r="A3" t="s">
         <v>113</v>
       </c>
@@ -22685,7 +22684,7 @@
         <v>374.820454719814</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" hidden="1" spans="1:3">
       <c r="A4" t="s">
         <v>45</v>
       </c>
@@ -22696,7 +22695,7 @@
         <v>266.652883320884</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" hidden="1" spans="1:3">
       <c r="A5" t="s">
         <v>46</v>
       </c>
@@ -22707,7 +22706,7 @@
         <v>278.438340293376</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" hidden="1" spans="1:3">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -22718,7 +22717,7 @@
         <v>256.272842595622</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" hidden="1" spans="1:3">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -22729,7 +22728,7 @@
         <v>266.286647805379</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" hidden="1" spans="1:3">
       <c r="A8" t="s">
         <v>114</v>
       </c>
@@ -22740,7 +22739,7 @@
         <v>262.094266831462</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" hidden="1" spans="1:3">
       <c r="A9" t="s">
         <v>97</v>
       </c>
@@ -22751,7 +22750,7 @@
         <v>301.862656296755</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" hidden="1" spans="1:3">
       <c r="A10" t="s">
         <v>115</v>
       </c>
@@ -22773,7 +22772,7 @@
         <v>301.301069854533</v>
       </c>
     </row>
-    <row r="12" spans="1:3">
+    <row r="12" hidden="1" spans="1:3">
       <c r="A12" t="s">
         <v>116</v>
       </c>
@@ -22784,7 +22783,7 @@
         <v>381.840985638718</v>
       </c>
     </row>
-    <row r="13" spans="1:3">
+    <row r="13" hidden="1" spans="1:3">
       <c r="A13" t="s">
         <v>117</v>
       </c>
@@ -22795,7 +22794,7 @@
         <v>340.965523745728</v>
       </c>
     </row>
-    <row r="14" spans="1:3">
+    <row r="14" hidden="1" spans="1:3">
       <c r="A14" t="s">
         <v>6</v>
       </c>
@@ -22806,7 +22805,7 @@
         <v>259.345063618978</v>
       </c>
     </row>
-    <row r="15" spans="1:3">
+    <row r="15" hidden="1" spans="1:3">
       <c r="A15" t="s">
         <v>118</v>
       </c>
@@ -22817,7 +22816,7 @@
         <v>222.249842950672</v>
       </c>
     </row>
-    <row r="16" spans="1:3">
+    <row r="16" hidden="1" spans="1:3">
       <c r="A16" t="s">
         <v>119</v>
       </c>
@@ -22828,7 +22827,7 @@
         <v>236.125508175659</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
+    <row r="17" hidden="1" spans="1:3">
       <c r="A17" t="s">
         <v>296</v>
       </c>
@@ -22839,7 +22838,7 @@
         <v>297.815210154215</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" hidden="1" spans="1:3">
       <c r="A18" t="s">
         <v>120</v>
       </c>
@@ -22850,7 +22849,7 @@
         <v>346.397011146938</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" hidden="1" spans="1:3">
       <c r="A19" t="s">
         <v>121</v>
       </c>
@@ -22861,7 +22860,7 @@
         <v>301.359587224325</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" hidden="1" spans="1:3">
       <c r="A20" t="s">
         <v>7</v>
       </c>
@@ -22872,7 +22871,7 @@
         <v>284.584019851685</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" hidden="1" spans="1:3">
       <c r="A21" t="s">
         <v>99</v>
       </c>
@@ -22883,7 +22882,7 @@
         <v>301.143964225815</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" hidden="1" spans="1:3">
       <c r="A22" t="s">
         <v>303</v>
       </c>
@@ -22894,7 +22893,7 @@
         <v>288.967370921202</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
+    <row r="23" hidden="1" spans="1:3">
       <c r="A23" t="s">
         <v>8</v>
       </c>
@@ -22905,7 +22904,7 @@
         <v>265.068741484782</v>
       </c>
     </row>
-    <row r="24" spans="1:3">
+    <row r="24" hidden="1" spans="1:3">
       <c r="A24" t="s">
         <v>311</v>
       </c>
@@ -22916,7 +22915,7 @@
         <v>295.906166832479</v>
       </c>
     </row>
-    <row r="25" spans="1:3">
+    <row r="25" hidden="1" spans="1:3">
       <c r="A25" t="s">
         <v>90</v>
       </c>
@@ -22949,7 +22948,7 @@
         <v>257.593297131551</v>
       </c>
     </row>
-    <row r="28" spans="1:3">
+    <row r="28" hidden="1" spans="1:3">
       <c r="A28" t="s">
         <v>47</v>
       </c>
@@ -22960,7 +22959,7 @@
         <v>324.435927186076</v>
       </c>
     </row>
-    <row r="29" spans="1:3">
+    <row r="29" hidden="1" spans="1:3">
       <c r="A29" t="s">
         <v>312</v>
       </c>
@@ -22971,7 +22970,7 @@
         <v>311.573719344451</v>
       </c>
     </row>
-    <row r="30" spans="1:3">
+    <row r="30" hidden="1" spans="1:3">
       <c r="A30" t="s">
         <v>122</v>
       </c>
@@ -22982,7 +22981,7 @@
         <v>334.820982196045</v>
       </c>
     </row>
-    <row r="31" spans="1:3">
+    <row r="31" hidden="1" spans="1:3">
       <c r="A31" t="s">
         <v>123</v>
       </c>
@@ -22993,7 +22992,7 @@
         <v>313.022724406501</v>
       </c>
     </row>
-    <row r="32" spans="1:3">
+    <row r="32" hidden="1" spans="1:3">
       <c r="A32" t="s">
         <v>124</v>
       </c>
@@ -23004,7 +23003,7 @@
         <v>255.742085797119</v>
       </c>
     </row>
-    <row r="33" spans="1:3">
+    <row r="33" hidden="1" spans="1:3">
       <c r="A33" t="s">
         <v>125</v>
       </c>
@@ -23015,7 +23014,7 @@
         <v>255.988960435384</v>
       </c>
     </row>
-    <row r="34" spans="1:3">
+    <row r="34" hidden="1" spans="1:3">
       <c r="A34" t="s">
         <v>9</v>
       </c>
@@ -23026,7 +23025,7 @@
         <v>292.718206883748</v>
       </c>
     </row>
-    <row r="35" spans="1:3">
+    <row r="35" hidden="1" spans="1:3">
       <c r="A35" t="s">
         <v>357</v>
       </c>
@@ -23037,7 +23036,7 @@
         <v>256.548239478992</v>
       </c>
     </row>
-    <row r="36" spans="1:3">
+    <row r="36" hidden="1" spans="1:3">
       <c r="A36" t="s">
         <v>48</v>
       </c>
@@ -23048,7 +23047,7 @@
         <v>293.897637628058</v>
       </c>
     </row>
-    <row r="37" spans="1:3">
+    <row r="37" hidden="1" spans="1:3">
       <c r="A37" t="s">
         <v>126</v>
       </c>
@@ -23059,7 +23058,7 @@
         <v>277.263542045811</v>
       </c>
     </row>
-    <row r="38" spans="1:3">
+    <row r="38" hidden="1" spans="1:3">
       <c r="A38" t="s">
         <v>49</v>
       </c>
@@ -23070,7 +23069,7 @@
         <v>286.019024036226</v>
       </c>
     </row>
-    <row r="39" spans="1:3">
+    <row r="39" hidden="1" spans="1:3">
       <c r="A39" t="s">
         <v>127</v>
       </c>
@@ -23081,7 +23080,7 @@
         <v>270.277655603027</v>
       </c>
     </row>
-    <row r="40" spans="1:3">
+    <row r="40" hidden="1" spans="1:3">
       <c r="A40" t="s">
         <v>128</v>
       </c>
@@ -23092,7 +23091,7 @@
         <v>219.242304530436</v>
       </c>
     </row>
-    <row r="41" spans="1:3">
+    <row r="41" hidden="1" spans="1:3">
       <c r="A41" t="s">
         <v>129</v>
       </c>
@@ -23103,7 +23102,7 @@
         <v>351.770519559326</v>
       </c>
     </row>
-    <row r="42" spans="1:3">
+    <row r="42" hidden="1" spans="1:3">
       <c r="A42" t="s">
         <v>130</v>
       </c>
@@ -23114,7 +23113,7 @@
         <v>433.876583432152</v>
       </c>
     </row>
-    <row r="43" spans="1:3">
+    <row r="43" hidden="1" spans="1:3">
       <c r="A43" t="s">
         <v>50</v>
       </c>
@@ -23125,7 +23124,7 @@
         <v>286.019024036226</v>
       </c>
     </row>
-    <row r="44" spans="1:3">
+    <row r="44" hidden="1" spans="1:3">
       <c r="A44" t="s">
         <v>131</v>
       </c>
@@ -23136,7 +23135,7 @@
         <v>241.516294023437</v>
       </c>
     </row>
-    <row r="45" spans="1:3">
+    <row r="45" hidden="1" spans="1:3">
       <c r="A45" t="s">
         <v>132</v>
       </c>
@@ -23147,7 +23146,7 @@
         <v>284.524463142904</v>
       </c>
     </row>
-    <row r="46" spans="1:3">
+    <row r="46" hidden="1" spans="1:3">
       <c r="A46" t="s">
         <v>351</v>
       </c>
@@ -23158,7 +23157,7 @@
         <v>326.77542401123</v>
       </c>
     </row>
-    <row r="47" spans="1:3">
+    <row r="47" hidden="1" spans="1:3">
       <c r="A47" t="s">
         <v>51</v>
       </c>
@@ -23169,7 +23168,7 @@
         <v>264.863844768609</v>
       </c>
     </row>
-    <row r="48" spans="1:3">
+    <row r="48" hidden="1" spans="1:3">
       <c r="A48" t="s">
         <v>91</v>
       </c>
@@ -23180,7 +23179,7 @@
         <v>283.656002196655</v>
       </c>
     </row>
-    <row r="49" spans="1:3">
+    <row r="49" hidden="1" spans="1:3">
       <c r="A49" t="s">
         <v>133</v>
       </c>
@@ -23191,7 +23190,7 @@
         <v>322.2152237854</v>
       </c>
     </row>
-    <row r="50" spans="1:3">
+    <row r="50" hidden="1" spans="1:3">
       <c r="A50" t="s">
         <v>134</v>
       </c>
@@ -23202,7 +23201,7 @@
         <v>357.15614496582</v>
       </c>
     </row>
-    <row r="51" spans="1:3">
+    <row r="51" hidden="1" spans="1:3">
       <c r="A51" t="s">
         <v>101</v>
       </c>
@@ -23213,7 +23212,7 @@
         <v>311.051468761916</v>
       </c>
     </row>
-    <row r="52" spans="1:3">
+    <row r="52" hidden="1" spans="1:3">
       <c r="A52" t="s">
         <v>135</v>
       </c>
@@ -23224,7 +23223,7 @@
         <v>285.279096714303</v>
       </c>
     </row>
-    <row r="53" spans="1:3">
+    <row r="53" hidden="1" spans="1:3">
       <c r="A53" t="s">
         <v>136</v>
       </c>
@@ -23235,7 +23234,7 @@
         <v>301.095322975667</v>
       </c>
     </row>
-    <row r="54" spans="1:3">
+    <row r="54" hidden="1" spans="1:3">
       <c r="A54" t="s">
         <v>313</v>
       </c>
@@ -23246,7 +23245,7 @@
         <v>311.573719344451</v>
       </c>
     </row>
-    <row r="55" spans="1:3">
+    <row r="55" hidden="1" spans="1:3">
       <c r="A55" t="s">
         <v>305</v>
       </c>
@@ -23257,7 +23256,7 @@
         <v>318.318822031657</v>
       </c>
     </row>
-    <row r="56" spans="1:3">
+    <row r="56" hidden="1" spans="1:3">
       <c r="A56" t="s">
         <v>137</v>
       </c>
@@ -23268,7 +23267,7 @@
         <v>304.131500134713</v>
       </c>
     </row>
-    <row r="57" spans="1:3">
+    <row r="57" hidden="1" spans="1:3">
       <c r="A57" t="s">
         <v>138</v>
       </c>
@@ -23279,7 +23278,7 @@
         <v>303.795792372105</v>
       </c>
     </row>
-    <row r="58" spans="1:3">
+    <row r="58" hidden="1" spans="1:3">
       <c r="A58" t="s">
         <v>102</v>
       </c>
@@ -23290,7 +23289,7 @@
         <v>312.001469702936</v>
       </c>
     </row>
-    <row r="59" spans="1:3">
+    <row r="59" hidden="1" spans="1:3">
       <c r="A59" t="s">
         <v>10</v>
       </c>
@@ -23301,7 +23300,7 @@
         <v>306.301368118286</v>
       </c>
     </row>
-    <row r="60" spans="1:3">
+    <row r="60" hidden="1" spans="1:3">
       <c r="A60" t="s">
         <v>139</v>
       </c>
@@ -23312,7 +23311,7 @@
         <v>357.759623572068</v>
       </c>
     </row>
-    <row r="61" spans="1:3">
+    <row r="61" hidden="1" spans="1:3">
       <c r="A61" t="s">
         <v>358</v>
       </c>
@@ -23334,7 +23333,7 @@
         <v>320.387998529188</v>
       </c>
     </row>
-    <row r="63" spans="1:3">
+    <row r="63" hidden="1" spans="1:3">
       <c r="A63" t="s">
         <v>141</v>
       </c>
@@ -23345,7 +23344,7 @@
         <v>279.35124236613</v>
       </c>
     </row>
-    <row r="64" spans="1:3">
+    <row r="64" hidden="1" spans="1:3">
       <c r="A64" t="s">
         <v>306</v>
       </c>
@@ -23356,7 +23355,7 @@
         <v>264.439106170509</v>
       </c>
     </row>
-    <row r="65" spans="1:3">
+    <row r="65" hidden="1" spans="1:3">
       <c r="A65" t="s">
         <v>11</v>
       </c>
@@ -23367,7 +23366,7 @@
         <v>342.956994409272</v>
       </c>
     </row>
-    <row r="66" spans="1:3">
+    <row r="66" hidden="1" spans="1:3">
       <c r="A66" t="s">
         <v>142</v>
       </c>
@@ -23378,7 +23377,7 @@
         <v>306.037306903483</v>
       </c>
     </row>
-    <row r="67" spans="1:3">
+    <row r="67" hidden="1" spans="1:3">
       <c r="A67" t="s">
         <v>314</v>
       </c>
@@ -23389,7 +23388,7 @@
         <v>317.778195477973</v>
       </c>
     </row>
-    <row r="68" spans="1:3">
+    <row r="68" hidden="1" spans="1:3">
       <c r="A68" t="s">
         <v>52</v>
       </c>
@@ -23400,7 +23399,7 @@
         <v>296.00326373759</v>
       </c>
     </row>
-    <row r="69" spans="1:3">
+    <row r="69" hidden="1" spans="1:3">
       <c r="A69" t="s">
         <v>315</v>
       </c>
@@ -23411,7 +23410,7 @@
         <v>322.687818957074</v>
       </c>
     </row>
-    <row r="70" spans="1:3">
+    <row r="70" hidden="1" spans="1:3">
       <c r="A70" t="s">
         <v>143</v>
       </c>
@@ -23422,7 +23421,7 @@
         <v>254.673271880086</v>
       </c>
     </row>
-    <row r="71" spans="1:3">
+    <row r="71" hidden="1" spans="1:3">
       <c r="A71" t="s">
         <v>53</v>
       </c>
@@ -23433,7 +23432,7 @@
         <v>266.652883320884</v>
       </c>
     </row>
-    <row r="72" spans="1:3">
+    <row r="72" hidden="1" spans="1:3">
       <c r="A72" t="s">
         <v>144</v>
       </c>
@@ -23444,7 +23443,7 @@
         <v>418.403982981364</v>
       </c>
     </row>
-    <row r="73" spans="1:3">
+    <row r="73" hidden="1" spans="1:3">
       <c r="A73" t="s">
         <v>12</v>
       </c>
@@ -23455,7 +23454,7 @@
         <v>287.831238739014</v>
       </c>
     </row>
-    <row r="74" spans="1:3">
+    <row r="74" hidden="1" spans="1:3">
       <c r="A74" t="s">
         <v>145</v>
       </c>
@@ -23466,7 +23465,7 @@
         <v>405.61251247142</v>
       </c>
     </row>
-    <row r="75" spans="1:3">
+    <row r="75" hidden="1" spans="1:3">
       <c r="A75" t="s">
         <v>13</v>
       </c>
@@ -23477,7 +23476,7 @@
         <v>302.665626832682</v>
       </c>
     </row>
-    <row r="76" spans="1:3">
+    <row r="76" hidden="1" spans="1:3">
       <c r="A76" t="s">
         <v>54</v>
       </c>
@@ -23488,7 +23487,7 @@
         <v>281.477843840826</v>
       </c>
     </row>
-    <row r="77" spans="1:3">
+    <row r="77" hidden="1" spans="1:3">
       <c r="A77" t="s">
         <v>146</v>
       </c>
@@ -23499,7 +23498,7 @@
         <v>335.613767778524</v>
       </c>
     </row>
-    <row r="78" spans="1:3">
+    <row r="78" hidden="1" spans="1:3">
       <c r="A78" t="s">
         <v>147</v>
       </c>
@@ -23510,7 +23509,7 @@
         <v>269.524066059803</v>
       </c>
     </row>
-    <row r="79" spans="1:3">
+    <row r="79" hidden="1" spans="1:3">
       <c r="A79" t="s">
         <v>148</v>
       </c>
@@ -23521,7 +23520,7 @@
         <v>320.706402989095</v>
       </c>
     </row>
-    <row r="80" spans="1:3">
+    <row r="80" hidden="1" spans="1:3">
       <c r="A80" t="s">
         <v>316</v>
       </c>
@@ -23532,7 +23531,7 @@
         <v>334.104775637139</v>
       </c>
     </row>
-    <row r="81" spans="1:3">
+    <row r="81" hidden="1" spans="1:3">
       <c r="A81" t="s">
         <v>149</v>
       </c>
@@ -23543,7 +23542,7 @@
         <v>328.078616319784</v>
       </c>
     </row>
-    <row r="82" spans="1:3">
+    <row r="82" hidden="1" spans="1:3">
       <c r="A82" t="s">
         <v>55</v>
       </c>
@@ -23554,7 +23553,7 @@
         <v>280.750138088989</v>
       </c>
     </row>
-    <row r="83" spans="1:3">
+    <row r="83" hidden="1" spans="1:3">
       <c r="A83" t="s">
         <v>56</v>
       </c>
@@ -23565,7 +23564,7 @@
         <v>327.962818049113</v>
       </c>
     </row>
-    <row r="84" spans="1:3">
+    <row r="84" hidden="1" spans="1:3">
       <c r="A84" t="s">
         <v>103</v>
       </c>
@@ -23576,7 +23575,7 @@
         <v>288.226014966779</v>
       </c>
     </row>
-    <row r="85" spans="1:3">
+    <row r="85" hidden="1" spans="1:3">
       <c r="A85" t="s">
         <v>14</v>
       </c>
@@ -23587,7 +23586,7 @@
         <v>263.010831723022</v>
       </c>
     </row>
-    <row r="86" spans="1:3">
+    <row r="86" hidden="1" spans="1:3">
       <c r="A86" t="s">
         <v>150</v>
       </c>
@@ -23598,7 +23597,7 @@
         <v>256.146674725545</v>
       </c>
     </row>
-    <row r="87" spans="1:3">
+    <row r="87" hidden="1" spans="1:3">
       <c r="A87" t="s">
         <v>151</v>
       </c>
@@ -23620,7 +23619,7 @@
         <v>312.423720951131</v>
       </c>
     </row>
-    <row r="89" spans="1:3">
+    <row r="89" hidden="1" spans="1:3">
       <c r="A89" t="s">
         <v>57</v>
       </c>
@@ -23631,7 +23630,7 @@
         <v>298.491834836426</v>
       </c>
     </row>
-    <row r="90" spans="1:3">
+    <row r="90" hidden="1" spans="1:3">
       <c r="A90" t="s">
         <v>317</v>
       </c>
@@ -23642,7 +23641,7 @@
         <v>311.536292573048</v>
       </c>
     </row>
-    <row r="91" spans="1:3">
+    <row r="91" hidden="1" spans="1:3">
       <c r="A91" t="s">
         <v>15</v>
       </c>
@@ -23653,7 +23652,7 @@
         <v>261.360629447632</v>
       </c>
     </row>
-    <row r="92" spans="1:3">
+    <row r="92" hidden="1" spans="1:3">
       <c r="A92" t="s">
         <v>58</v>
       </c>
@@ -23664,7 +23663,7 @@
         <v>266.162307542637</v>
       </c>
     </row>
-    <row r="93" spans="1:3">
+    <row r="93" hidden="1" spans="1:3">
       <c r="A93" t="s">
         <v>16</v>
       </c>
@@ -23675,7 +23674,7 @@
         <v>298.610538777669</v>
       </c>
     </row>
-    <row r="94" spans="1:3">
+    <row r="94" hidden="1" spans="1:3">
       <c r="A94" t="s">
         <v>59</v>
       </c>
@@ -23686,7 +23685,7 @@
         <v>288.255788633219</v>
       </c>
     </row>
-    <row r="95" spans="1:3">
+    <row r="95" hidden="1" spans="1:3">
       <c r="A95" t="s">
         <v>153</v>
       </c>
@@ -23697,7 +23696,7 @@
         <v>261.008269402262</v>
       </c>
     </row>
-    <row r="96" spans="1:3">
+    <row r="96" hidden="1" spans="1:3">
       <c r="A96" t="s">
         <v>60</v>
       </c>
@@ -23708,7 +23707,7 @@
         <v>306.353868303426</v>
       </c>
     </row>
-    <row r="97" spans="1:3">
+    <row r="97" hidden="1" spans="1:3">
       <c r="A97" t="s">
         <v>154</v>
       </c>
@@ -23719,7 +23718,7 @@
         <v>290.696817822266</v>
       </c>
     </row>
-    <row r="98" spans="1:3">
+    <row r="98" hidden="1" spans="1:3">
       <c r="A98" t="s">
         <v>359</v>
       </c>
@@ -23730,7 +23729,7 @@
         <v>255.674141887411</v>
       </c>
     </row>
-    <row r="99" spans="1:3">
+    <row r="99" hidden="1" spans="1:3">
       <c r="A99" t="s">
         <v>155</v>
       </c>
@@ -23741,7 +23740,7 @@
         <v>228.105133128459</v>
       </c>
     </row>
-    <row r="100" spans="1:3">
+    <row r="100" hidden="1" spans="1:3">
       <c r="A100" t="s">
         <v>348</v>
       </c>
@@ -23752,7 +23751,7 @@
         <v>354.961474793585</v>
       </c>
     </row>
-    <row r="101" spans="1:3">
+    <row r="101" hidden="1" spans="1:3">
       <c r="A101" t="s">
         <v>104</v>
       </c>
@@ -23763,7 +23762,7 @@
         <v>252.047301495256</v>
       </c>
     </row>
-    <row r="102" spans="1:3">
+    <row r="102" hidden="1" spans="1:3">
       <c r="A102" t="s">
         <v>61</v>
       </c>
@@ -23774,7 +23773,7 @@
         <v>279.525451658994</v>
       </c>
     </row>
-    <row r="103" spans="1:3">
+    <row r="103" hidden="1" spans="1:3">
       <c r="A103" t="s">
         <v>360</v>
       </c>
@@ -23785,7 +23784,7 @@
         <v>257.15623451199</v>
       </c>
     </row>
-    <row r="104" spans="1:3">
+    <row r="104" hidden="1" spans="1:3">
       <c r="A104" t="s">
         <v>349</v>
       </c>
@@ -23796,7 +23795,7 @@
         <v>315.614844885254</v>
       </c>
     </row>
-    <row r="105" spans="1:3">
+    <row r="105" hidden="1" spans="1:3">
       <c r="A105" t="s">
         <v>17</v>
       </c>
@@ -23807,7 +23806,7 @@
         <v>347.628001876831</v>
       </c>
     </row>
-    <row r="106" spans="1:3">
+    <row r="106" hidden="1" spans="1:3">
       <c r="A106" t="s">
         <v>318</v>
       </c>
@@ -23818,7 +23817,7 @@
         <v>311.573719344451</v>
       </c>
     </row>
-    <row r="107" spans="1:3">
+    <row r="107" hidden="1" spans="1:3">
       <c r="A107" t="s">
         <v>156</v>
       </c>
@@ -23829,7 +23828,7 @@
         <v>271.918151871047</v>
       </c>
     </row>
-    <row r="108" spans="1:3">
+    <row r="108" hidden="1" spans="1:3">
       <c r="A108" t="s">
         <v>157</v>
       </c>
@@ -23840,7 +23839,7 @@
         <v>224.784511560059</v>
       </c>
     </row>
-    <row r="109" spans="1:3">
+    <row r="109" hidden="1" spans="1:3">
       <c r="A109" t="s">
         <v>62</v>
       </c>
@@ -23851,7 +23850,7 @@
         <v>241.034410733032</v>
       </c>
     </row>
-    <row r="110" spans="1:3">
+    <row r="110" hidden="1" spans="1:3">
       <c r="A110" t="s">
         <v>63</v>
       </c>
@@ -23873,7 +23872,7 @@
         <v>274.629233492461</v>
       </c>
     </row>
-    <row r="112" spans="1:3">
+    <row r="112" hidden="1" spans="1:3">
       <c r="A112" t="s">
         <v>158</v>
       </c>
@@ -23884,7 +23883,7 @@
         <v>406.444289532761</v>
       </c>
     </row>
-    <row r="113" spans="1:3">
+    <row r="113" hidden="1" spans="1:3">
       <c r="A113" t="s">
         <v>18</v>
       </c>
@@ -23895,7 +23894,7 @@
         <v>259.659329971314</v>
       </c>
     </row>
-    <row r="114" spans="1:3">
+    <row r="114" hidden="1" spans="1:3">
       <c r="A114" t="s">
         <v>319</v>
       </c>
@@ -23906,7 +23905,7 @@
         <v>296.587988627116</v>
       </c>
     </row>
-    <row r="115" spans="1:3">
+    <row r="115" hidden="1" spans="1:3">
       <c r="A115" t="s">
         <v>361</v>
       </c>
@@ -23917,7 +23916,7 @@
         <v>268.648630470785</v>
       </c>
     </row>
-    <row r="116" spans="1:3">
+    <row r="116" hidden="1" spans="1:3">
       <c r="A116" t="s">
         <v>64</v>
       </c>
@@ -23928,7 +23927,7 @@
         <v>309.027064755046</v>
       </c>
     </row>
-    <row r="117" spans="1:3">
+    <row r="117" hidden="1" spans="1:3">
       <c r="A117" t="s">
         <v>159</v>
       </c>
@@ -23939,7 +23938,7 @@
         <v>321.682966754761</v>
       </c>
     </row>
-    <row r="118" spans="1:3">
+    <row r="118" hidden="1" spans="1:3">
       <c r="A118" t="s">
         <v>19</v>
       </c>
@@ -23950,7 +23949,7 @@
         <v>279.028359132313</v>
       </c>
     </row>
-    <row r="119" spans="1:3">
+    <row r="119" hidden="1" spans="1:3">
       <c r="A119" t="s">
         <v>160</v>
       </c>
@@ -23961,7 +23960,7 @@
         <v>271.918151871047</v>
       </c>
     </row>
-    <row r="120" spans="1:3">
+    <row r="120" hidden="1" spans="1:3">
       <c r="A120" t="s">
         <v>161</v>
       </c>
@@ -23972,7 +23971,7 @@
         <v>381.840985638718</v>
       </c>
     </row>
-    <row r="121" spans="1:3">
+    <row r="121" hidden="1" spans="1:3">
       <c r="A121" t="s">
         <v>65</v>
       </c>
@@ -23983,7 +23982,7 @@
         <v>295.596061356637</v>
       </c>
     </row>
-    <row r="122" spans="1:3">
+    <row r="122" hidden="1" spans="1:3">
       <c r="A122" t="s">
         <v>66</v>
       </c>
@@ -23994,7 +23993,7 @@
         <v>258.312873334525</v>
       </c>
     </row>
-    <row r="123" spans="1:3">
+    <row r="123" hidden="1" spans="1:3">
       <c r="A123" t="s">
         <v>162</v>
       </c>
@@ -24005,7 +24004,7 @@
         <v>222.761283909709</v>
       </c>
     </row>
-    <row r="124" spans="1:3">
+    <row r="124" hidden="1" spans="1:3">
       <c r="A124" t="s">
         <v>320</v>
       </c>
@@ -24016,7 +24015,7 @@
         <v>317.778195477973</v>
       </c>
     </row>
-    <row r="125" spans="1:3">
+    <row r="125" hidden="1" spans="1:3">
       <c r="A125" t="s">
         <v>163</v>
       </c>
@@ -24027,7 +24026,7 @@
         <v>283.993054762777</v>
       </c>
     </row>
-    <row r="126" spans="1:3">
+    <row r="126" hidden="1" spans="1:3">
       <c r="A126" t="s">
         <v>105</v>
       </c>
@@ -24038,7 +24037,7 @@
         <v>313.853176361956</v>
       </c>
     </row>
-    <row r="127" spans="1:3">
+    <row r="127" hidden="1" spans="1:3">
       <c r="A127" t="s">
         <v>164</v>
       </c>
@@ -24049,7 +24048,7 @@
         <v>272.92370219808</v>
       </c>
     </row>
-    <row r="128" spans="1:3">
+    <row r="128" hidden="1" spans="1:3">
       <c r="A128" t="s">
         <v>165</v>
       </c>
@@ -24071,7 +24070,7 @@
         <v>359.541413859049</v>
       </c>
     </row>
-    <row r="130" spans="1:3">
+    <row r="130" hidden="1" spans="1:3">
       <c r="A130" t="s">
         <v>167</v>
       </c>
@@ -24082,7 +24081,7 @@
         <v>397.924830148185</v>
       </c>
     </row>
-    <row r="131" spans="1:3">
+    <row r="131" hidden="1" spans="1:3">
       <c r="A131" t="s">
         <v>362</v>
       </c>
@@ -24093,7 +24092,7 @@
         <v>381.909496512858</v>
       </c>
     </row>
-    <row r="132" spans="1:3">
+    <row r="132" hidden="1" spans="1:3">
       <c r="A132" t="s">
         <v>321</v>
       </c>
@@ -24104,7 +24103,7 @@
         <v>290.399983863525</v>
       </c>
     </row>
-    <row r="133" spans="1:3">
+    <row r="133" hidden="1" spans="1:3">
       <c r="A133" t="s">
         <v>168</v>
       </c>
@@ -24115,7 +24114,7 @@
         <v>296.954669174194</v>
       </c>
     </row>
-    <row r="134" spans="1:3">
+    <row r="134" hidden="1" spans="1:3">
       <c r="A134" t="s">
         <v>169</v>
       </c>
@@ -24126,7 +24125,7 @@
         <v>309.253734095459</v>
       </c>
     </row>
-    <row r="135" spans="1:3">
+    <row r="135" hidden="1" spans="1:3">
       <c r="A135" t="s">
         <v>170</v>
       </c>
@@ -24137,7 +24136,7 @@
         <v>321.928933681234</v>
       </c>
     </row>
-    <row r="136" spans="1:3">
+    <row r="136" hidden="1" spans="1:3">
       <c r="A136" t="s">
         <v>171</v>
       </c>
@@ -24148,7 +24147,7 @@
         <v>203.805663054403</v>
       </c>
     </row>
-    <row r="137" spans="1:3">
+    <row r="137" hidden="1" spans="1:3">
       <c r="A137" t="s">
         <v>172</v>
       </c>
@@ -24159,7 +24158,7 @@
         <v>196.826176896973</v>
       </c>
     </row>
-    <row r="138" spans="1:3">
+    <row r="138" hidden="1" spans="1:3">
       <c r="A138" t="s">
         <v>173</v>
       </c>
@@ -24170,7 +24169,7 @@
         <v>259.910897463989</v>
       </c>
     </row>
-    <row r="139" spans="1:3">
+    <row r="139" hidden="1" spans="1:3">
       <c r="A139" t="s">
         <v>174</v>
       </c>
@@ -24181,7 +24180,7 @@
         <v>415.947517088523</v>
       </c>
     </row>
-    <row r="140" spans="1:3">
+    <row r="140" hidden="1" spans="1:3">
       <c r="A140" t="s">
         <v>175</v>
       </c>
@@ -24192,7 +24191,7 @@
         <v>374.820454719814</v>
       </c>
     </row>
-    <row r="141" spans="1:3">
+    <row r="141" hidden="1" spans="1:3">
       <c r="A141" t="s">
         <v>176</v>
       </c>
@@ -24203,7 +24202,7 @@
         <v>388.890601956458</v>
       </c>
     </row>
-    <row r="142" spans="1:3">
+    <row r="142" hidden="1" spans="1:3">
       <c r="A142" t="s">
         <v>177</v>
       </c>
@@ -24214,7 +24213,7 @@
         <v>365.675141665039</v>
       </c>
     </row>
-    <row r="143" spans="1:3">
+    <row r="143" hidden="1" spans="1:3">
       <c r="A143" t="s">
         <v>178</v>
       </c>
@@ -24225,7 +24224,7 @@
         <v>371.812812164307</v>
       </c>
     </row>
-    <row r="144" spans="1:3">
+    <row r="144" hidden="1" spans="1:3">
       <c r="A144" t="s">
         <v>179</v>
       </c>
@@ -24247,7 +24246,7 @@
         <v>305.000461785997</v>
       </c>
     </row>
-    <row r="146" spans="1:3">
+    <row r="146" hidden="1" spans="1:3">
       <c r="A146" t="s">
         <v>180</v>
       </c>
@@ -24258,7 +24257,7 @@
         <v>397.013463482666</v>
       </c>
     </row>
-    <row r="147" spans="1:3">
+    <row r="147" hidden="1" spans="1:3">
       <c r="A147" t="s">
         <v>297</v>
       </c>
@@ -24269,7 +24268,7 @@
         <v>294.172829421997</v>
       </c>
     </row>
-    <row r="148" spans="1:3">
+    <row r="148" hidden="1" spans="1:3">
       <c r="A148" t="s">
         <v>20</v>
       </c>
@@ -24291,7 +24290,7 @@
         <v>323.653923058065</v>
       </c>
     </row>
-    <row r="150" spans="1:3">
+    <row r="150" hidden="1" spans="1:3">
       <c r="A150" t="s">
         <v>182</v>
       </c>
@@ -24313,7 +24312,7 @@
         <v>323.675307876587</v>
       </c>
     </row>
-    <row r="152" spans="1:3">
+    <row r="152" hidden="1" spans="1:3">
       <c r="A152" t="s">
         <v>184</v>
       </c>
@@ -24324,7 +24323,7 @@
         <v>335.648423689662</v>
       </c>
     </row>
-    <row r="153" spans="1:3">
+    <row r="153" hidden="1" spans="1:3">
       <c r="A153" t="s">
         <v>21</v>
       </c>
@@ -24335,7 +24334,7 @@
         <v>294.602864461176</v>
       </c>
     </row>
-    <row r="154" spans="1:3">
+    <row r="154" hidden="1" spans="1:3">
       <c r="A154" t="s">
         <v>185</v>
       </c>
@@ -24346,7 +24345,7 @@
         <v>358.261246794434</v>
       </c>
     </row>
-    <row r="155" spans="1:3">
+    <row r="155" hidden="1" spans="1:3">
       <c r="A155" t="s">
         <v>22</v>
       </c>
@@ -24368,7 +24367,7 @@
         <v>278.613505499897</v>
       </c>
     </row>
-    <row r="157" spans="1:3">
+    <row r="157" hidden="1" spans="1:3">
       <c r="A157" t="s">
         <v>186</v>
       </c>
@@ -24379,7 +24378,7 @@
         <v>229.620712825811</v>
       </c>
     </row>
-    <row r="158" spans="1:3">
+    <row r="158" hidden="1" spans="1:3">
       <c r="A158" t="s">
         <v>363</v>
       </c>
@@ -24390,7 +24389,7 @@
         <v>336.047785916748</v>
       </c>
     </row>
-    <row r="159" spans="1:3">
+    <row r="159" hidden="1" spans="1:3">
       <c r="A159" t="s">
         <v>23</v>
       </c>
@@ -24401,7 +24400,7 @@
         <v>263.010831723022</v>
       </c>
     </row>
-    <row r="160" spans="1:3">
+    <row r="160" hidden="1" spans="1:3">
       <c r="A160" t="s">
         <v>3</v>
       </c>
@@ -24423,7 +24422,7 @@
         <v>350.530375691325</v>
       </c>
     </row>
-    <row r="162" spans="1:3">
+    <row r="162" hidden="1" spans="1:3">
       <c r="A162" t="s">
         <v>188</v>
       </c>
@@ -24434,7 +24433,7 @@
         <v>263.355220677926</v>
       </c>
     </row>
-    <row r="163" spans="1:3">
+    <row r="163" hidden="1" spans="1:3">
       <c r="A163" t="s">
         <v>92</v>
       </c>
@@ -24456,7 +24455,7 @@
         <v>336.189021045212</v>
       </c>
     </row>
-    <row r="165" spans="1:3">
+    <row r="165" hidden="1" spans="1:3">
       <c r="A165" t="s">
         <v>24</v>
       </c>
@@ -24467,7 +24466,7 @@
         <v>239.226625744832</v>
       </c>
     </row>
-    <row r="166" spans="1:3">
+    <row r="166" hidden="1" spans="1:3">
       <c r="A166" t="s">
         <v>189</v>
       </c>
@@ -24478,7 +24477,7 @@
         <v>335.265040920003</v>
       </c>
     </row>
-    <row r="167" spans="1:3">
+    <row r="167" hidden="1" spans="1:3">
       <c r="A167" t="s">
         <v>67</v>
       </c>
@@ -24489,7 +24488,7 @@
         <v>298.774593423462</v>
       </c>
     </row>
-    <row r="168" spans="1:3">
+    <row r="168" hidden="1" spans="1:3">
       <c r="A168" t="s">
         <v>25</v>
       </c>
@@ -24500,7 +24499,7 @@
         <v>300.830686157227</v>
       </c>
     </row>
-    <row r="169" spans="1:3">
+    <row r="169" hidden="1" spans="1:3">
       <c r="A169" t="s">
         <v>325</v>
       </c>
@@ -24522,7 +24521,7 @@
         <v>313.224918787009</v>
       </c>
     </row>
-    <row r="171" spans="1:3">
+    <row r="171" hidden="1" spans="1:3">
       <c r="A171" t="s">
         <v>191</v>
       </c>
@@ -24533,7 +24532,7 @@
         <v>240.385434202677</v>
       </c>
     </row>
-    <row r="172" spans="1:3">
+    <row r="172" hidden="1" spans="1:3">
       <c r="A172" t="s">
         <v>192</v>
       </c>
@@ -24544,7 +24543,7 @@
         <v>241.098204802653</v>
       </c>
     </row>
-    <row r="173" spans="1:3">
+    <row r="173" hidden="1" spans="1:3">
       <c r="A173" t="s">
         <v>193</v>
       </c>
@@ -24555,7 +24554,7 @@
         <v>208.067991691894</v>
       </c>
     </row>
-    <row r="174" spans="1:3">
+    <row r="174" hidden="1" spans="1:3">
       <c r="A174" t="s">
         <v>364</v>
       </c>
@@ -24566,7 +24565,7 @@
         <v>260.174123518299</v>
       </c>
     </row>
-    <row r="175" spans="1:3">
+    <row r="175" hidden="1" spans="1:3">
       <c r="A175" t="s">
         <v>194</v>
       </c>
@@ -24588,7 +24587,7 @@
         <v>338.275968037923</v>
       </c>
     </row>
-    <row r="177" spans="1:3">
+    <row r="177" hidden="1" spans="1:3">
       <c r="A177" t="s">
         <v>196</v>
       </c>
@@ -24599,7 +24598,7 @@
         <v>214.219092605591</v>
       </c>
     </row>
-    <row r="178" spans="1:3">
+    <row r="178" hidden="1" spans="1:3">
       <c r="A178" t="s">
         <v>197</v>
       </c>
@@ -24610,7 +24609,7 @@
         <v>333.010537028808</v>
       </c>
     </row>
-    <row r="179" spans="1:3">
+    <row r="179" hidden="1" spans="1:3">
       <c r="A179" t="s">
         <v>198</v>
       </c>
@@ -24621,7 +24620,7 @@
         <v>233.608455651245</v>
       </c>
     </row>
-    <row r="180" spans="1:3">
+    <row r="180" hidden="1" spans="1:3">
       <c r="A180" t="s">
         <v>326</v>
       </c>
@@ -24632,7 +24631,7 @@
         <v>278.757855618625</v>
       </c>
     </row>
-    <row r="181" spans="1:3">
+    <row r="181" hidden="1" spans="1:3">
       <c r="A181" t="s">
         <v>106</v>
       </c>
@@ -24654,7 +24653,7 @@
         <v>294.705919165911</v>
       </c>
     </row>
-    <row r="183" spans="1:3">
+    <row r="183" hidden="1" spans="1:3">
       <c r="A183" t="s">
         <v>199</v>
       </c>
@@ -24665,7 +24664,7 @@
         <v>251.383093243408</v>
       </c>
     </row>
-    <row r="184" spans="1:3">
+    <row r="184" hidden="1" spans="1:3">
       <c r="A184" t="s">
         <v>200</v>
       </c>
@@ -24676,7 +24675,7 @@
         <v>229.815356249961</v>
       </c>
     </row>
-    <row r="185" spans="1:3">
+    <row r="185" hidden="1" spans="1:3">
       <c r="A185" t="s">
         <v>26</v>
       </c>
@@ -24698,7 +24697,7 @@
         <v>289.770245502521</v>
       </c>
     </row>
-    <row r="187" spans="1:3">
+    <row r="187" hidden="1" spans="1:3">
       <c r="A187" t="s">
         <v>327</v>
       </c>
@@ -24709,7 +24708,7 @@
         <v>278.22761177063</v>
       </c>
     </row>
-    <row r="188" spans="1:3">
+    <row r="188" hidden="1" spans="1:3">
       <c r="A188" t="s">
         <v>202</v>
       </c>
@@ -24720,7 +24719,7 @@
         <v>465.451525565011</v>
       </c>
     </row>
-    <row r="189" spans="1:3">
+    <row r="189" hidden="1" spans="1:3">
       <c r="A189" t="s">
         <v>203</v>
       </c>
@@ -24742,7 +24741,7 @@
         <v>305.131214928618</v>
       </c>
     </row>
-    <row r="191" spans="1:3">
+    <row r="191" hidden="1" spans="1:3">
       <c r="A191" t="s">
         <v>69</v>
       </c>
@@ -24753,7 +24752,7 @@
         <v>321.059078714193</v>
       </c>
     </row>
-    <row r="192" spans="1:3">
+    <row r="192" hidden="1" spans="1:3">
       <c r="A192" t="s">
         <v>205</v>
       </c>
@@ -24764,7 +24763,7 @@
         <v>279.368847271118</v>
       </c>
     </row>
-    <row r="193" spans="1:3">
+    <row r="193" hidden="1" spans="1:3">
       <c r="A193" t="s">
         <v>206</v>
       </c>
@@ -24775,7 +24774,7 @@
         <v>232.539638578898</v>
       </c>
     </row>
-    <row r="194" spans="1:3">
+    <row r="194" hidden="1" spans="1:3">
       <c r="A194" t="s">
         <v>207</v>
       </c>
@@ -24786,7 +24785,7 @@
         <v>403.331082918701</v>
       </c>
     </row>
-    <row r="195" spans="1:3">
+    <row r="195" hidden="1" spans="1:3">
       <c r="A195" t="s">
         <v>208</v>
       </c>
@@ -24808,7 +24807,7 @@
         <v>304.351106987508</v>
       </c>
     </row>
-    <row r="197" spans="1:3">
+    <row r="197" hidden="1" spans="1:3">
       <c r="A197" t="s">
         <v>329</v>
       </c>
@@ -24819,7 +24818,7 @@
         <v>287.472536399429</v>
       </c>
     </row>
-    <row r="198" spans="1:3">
+    <row r="198" hidden="1" spans="1:3">
       <c r="A198" t="s">
         <v>352</v>
       </c>
@@ -24830,7 +24829,7 @@
         <v>324.859061691284</v>
       </c>
     </row>
-    <row r="199" spans="1:3">
+    <row r="199" hidden="1" spans="1:3">
       <c r="A199" t="s">
         <v>27</v>
       </c>
@@ -24841,7 +24840,7 @@
         <v>300.66894881307</v>
       </c>
     </row>
-    <row r="200" spans="1:3">
+    <row r="200" hidden="1" spans="1:3">
       <c r="A200" t="s">
         <v>330</v>
       </c>
@@ -24852,7 +24851,7 @@
         <v>278.757855618625</v>
       </c>
     </row>
-    <row r="201" spans="1:3">
+    <row r="201" hidden="1" spans="1:3">
       <c r="A201" t="s">
         <v>70</v>
       </c>
@@ -24863,7 +24862,7 @@
         <v>279.25530979716</v>
       </c>
     </row>
-    <row r="202" spans="1:3">
+    <row r="202" hidden="1" spans="1:3">
       <c r="A202" t="s">
         <v>365</v>
       </c>
@@ -24874,7 +24873,7 @@
         <v>267.710740955549</v>
       </c>
     </row>
-    <row r="203" spans="1:3">
+    <row r="203" hidden="1" spans="1:3">
       <c r="A203" t="s">
         <v>209</v>
       </c>
@@ -24885,7 +24884,7 @@
         <v>285.931365398966</v>
       </c>
     </row>
-    <row r="204" spans="1:3">
+    <row r="204" hidden="1" spans="1:3">
       <c r="A204" t="s">
         <v>210</v>
       </c>
@@ -24896,7 +24895,7 @@
         <v>241.979724950968</v>
       </c>
     </row>
-    <row r="205" spans="1:3">
+    <row r="205" hidden="1" spans="1:3">
       <c r="A205" t="s">
         <v>71</v>
       </c>
@@ -24907,7 +24906,7 @@
         <v>279.525451658994</v>
       </c>
     </row>
-    <row r="206" spans="1:3">
+    <row r="206" hidden="1" spans="1:3">
       <c r="A206" t="s">
         <v>211</v>
       </c>
@@ -24918,7 +24917,7 @@
         <v>264.760615571086</v>
       </c>
     </row>
-    <row r="207" spans="1:3">
+    <row r="207" hidden="1" spans="1:3">
       <c r="A207" t="s">
         <v>212</v>
       </c>
@@ -24929,7 +24928,7 @@
         <v>313.523703348999</v>
       </c>
     </row>
-    <row r="208" spans="1:3">
+    <row r="208" hidden="1" spans="1:3">
       <c r="A208" t="s">
         <v>213</v>
       </c>
@@ -24940,7 +24939,7 @@
         <v>234.091338290958</v>
       </c>
     </row>
-    <row r="209" spans="1:3">
+    <row r="209" hidden="1" spans="1:3">
       <c r="A209" t="s">
         <v>214</v>
       </c>
@@ -24951,7 +24950,7 @@
         <v>257.393929834798</v>
       </c>
     </row>
-    <row r="210" spans="1:3">
+    <row r="210" hidden="1" spans="1:3">
       <c r="A210" t="s">
         <v>215</v>
       </c>
@@ -24962,7 +24961,7 @@
         <v>362.332862310791</v>
       </c>
     </row>
-    <row r="211" spans="1:3">
+    <row r="211" hidden="1" spans="1:3">
       <c r="A211" t="s">
         <v>216</v>
       </c>
@@ -24973,7 +24972,7 @@
         <v>437.172851081485</v>
       </c>
     </row>
-    <row r="212" spans="1:3">
+    <row r="212" hidden="1" spans="1:3">
       <c r="A212" t="s">
         <v>331</v>
       </c>
@@ -24984,7 +24983,7 @@
         <v>295.945580834961</v>
       </c>
     </row>
-    <row r="213" spans="1:3">
+    <row r="213" hidden="1" spans="1:3">
       <c r="A213" t="s">
         <v>217</v>
       </c>
@@ -24995,7 +24994,7 @@
         <v>369.649409275309</v>
       </c>
     </row>
-    <row r="214" spans="1:3">
+    <row r="214" hidden="1" spans="1:3">
       <c r="A214" t="s">
         <v>218</v>
       </c>
@@ -25006,7 +25005,7 @@
         <v>216.545839467163</v>
       </c>
     </row>
-    <row r="215" spans="1:3">
+    <row r="215" hidden="1" spans="1:3">
       <c r="A215" t="s">
         <v>219</v>
       </c>
@@ -25017,7 +25016,7 @@
         <v>378.827240008545</v>
       </c>
     </row>
-    <row r="216" spans="1:3">
+    <row r="216" hidden="1" spans="1:3">
       <c r="A216" t="s">
         <v>220</v>
       </c>
@@ -25028,7 +25027,7 @@
         <v>343.426359114583</v>
       </c>
     </row>
-    <row r="217" spans="1:3">
+    <row r="217" hidden="1" spans="1:3">
       <c r="A217" t="s">
         <v>332</v>
       </c>
@@ -25039,7 +25038,7 @@
         <v>301.176327819824</v>
       </c>
     </row>
-    <row r="218" spans="1:3">
+    <row r="218" hidden="1" spans="1:3">
       <c r="A218" t="s">
         <v>221</v>
       </c>
@@ -25050,7 +25049,7 @@
         <v>415.947517088523</v>
       </c>
     </row>
-    <row r="219" spans="1:3">
+    <row r="219" hidden="1" spans="1:3">
       <c r="A219" t="s">
         <v>93</v>
       </c>
@@ -25061,7 +25060,7 @@
         <v>287.939654536743</v>
       </c>
     </row>
-    <row r="220" spans="1:3">
+    <row r="220" hidden="1" spans="1:3">
       <c r="A220" t="s">
         <v>72</v>
       </c>
@@ -25072,7 +25071,7 @@
         <v>255.520468488469</v>
       </c>
     </row>
-    <row r="221" spans="1:3">
+    <row r="221" hidden="1" spans="1:3">
       <c r="A221" t="s">
         <v>28</v>
       </c>
@@ -25083,7 +25082,7 @@
         <v>306.637912806193</v>
       </c>
     </row>
-    <row r="222" spans="1:3">
+    <row r="222" hidden="1" spans="1:3">
       <c r="A222" t="s">
         <v>222</v>
       </c>
@@ -25116,7 +25115,7 @@
         <v>353.804843592936</v>
       </c>
     </row>
-    <row r="225" spans="1:3">
+    <row r="225" hidden="1" spans="1:3">
       <c r="A225" t="s">
         <v>224</v>
       </c>
@@ -25138,7 +25137,7 @@
         <v>354.657285651042</v>
       </c>
     </row>
-    <row r="227" spans="1:3">
+    <row r="227" hidden="1" spans="1:3">
       <c r="A227" t="s">
         <v>73</v>
       </c>
@@ -25160,7 +25159,7 @@
         <v>298.801030088734</v>
       </c>
     </row>
-    <row r="229" spans="1:3">
+    <row r="229" hidden="1" spans="1:3">
       <c r="A229" t="s">
         <v>353</v>
       </c>
@@ -25171,7 +25170,7 @@
         <v>260.543137390137</v>
       </c>
     </row>
-    <row r="230" spans="1:3">
+    <row r="230" hidden="1" spans="1:3">
       <c r="A230" t="s">
         <v>226</v>
       </c>
@@ -25182,7 +25181,7 @@
         <v>164.700392940877</v>
       </c>
     </row>
-    <row r="231" spans="1:3">
+    <row r="231" hidden="1" spans="1:3">
       <c r="A231" t="s">
         <v>366</v>
       </c>
@@ -25193,7 +25192,7 @@
         <v>260.798229663696</v>
       </c>
     </row>
-    <row r="232" spans="1:3">
+    <row r="232" hidden="1" spans="1:3">
       <c r="A232" t="s">
         <v>74</v>
       </c>
@@ -25204,7 +25203,7 @@
         <v>285.558036512248</v>
       </c>
     </row>
-    <row r="233" spans="1:3">
+    <row r="233" hidden="1" spans="1:3">
       <c r="A233" t="s">
         <v>335</v>
       </c>
@@ -25215,7 +25214,7 @@
         <v>301.623879252116</v>
       </c>
     </row>
-    <row r="234" spans="1:3">
+    <row r="234" hidden="1" spans="1:3">
       <c r="A234" t="s">
         <v>336</v>
       </c>
@@ -25226,7 +25225,7 @@
         <v>299.453939961703</v>
       </c>
     </row>
-    <row r="235" spans="1:3">
+    <row r="235" hidden="1" spans="1:3">
       <c r="A235" t="s">
         <v>354</v>
       </c>
@@ -25248,7 +25247,7 @@
         <v>388.385146406139</v>
       </c>
     </row>
-    <row r="237" spans="1:3">
+    <row r="237" hidden="1" spans="1:3">
       <c r="A237" t="s">
         <v>107</v>
       </c>
@@ -25259,7 +25258,7 @@
         <v>316.067287884236</v>
       </c>
     </row>
-    <row r="238" spans="1:3">
+    <row r="238" hidden="1" spans="1:3">
       <c r="A238" t="s">
         <v>228</v>
       </c>
@@ -25270,7 +25269,7 @@
         <v>342.412460681966</v>
       </c>
     </row>
-    <row r="239" spans="1:3">
+    <row r="239" hidden="1" spans="1:3">
       <c r="A239" t="s">
         <v>75</v>
       </c>
@@ -25281,7 +25280,7 @@
         <v>273.484921468099</v>
       </c>
     </row>
-    <row r="240" spans="1:3">
+    <row r="240" hidden="1" spans="1:3">
       <c r="A240" t="s">
         <v>367</v>
       </c>
@@ -25292,7 +25291,7 @@
         <v>209.139593682658</v>
       </c>
     </row>
-    <row r="241" spans="1:3">
+    <row r="241" hidden="1" spans="1:3">
       <c r="A241" t="s">
         <v>229</v>
       </c>
@@ -25303,7 +25302,7 @@
         <v>280.080248683675</v>
       </c>
     </row>
-    <row r="242" spans="1:3">
+    <row r="242" hidden="1" spans="1:3">
       <c r="A242" t="s">
         <v>76</v>
       </c>
@@ -25314,7 +25313,7 @@
         <v>296.00326373759</v>
       </c>
     </row>
-    <row r="243" spans="1:3">
+    <row r="243" hidden="1" spans="1:3">
       <c r="A243" t="s">
         <v>308</v>
       </c>
@@ -25325,7 +25324,7 @@
         <v>282.864422478667</v>
       </c>
     </row>
-    <row r="244" spans="1:3">
+    <row r="244" hidden="1" spans="1:3">
       <c r="A244" t="s">
         <v>29</v>
       </c>
@@ -25336,7 +25335,7 @@
         <v>306.119932551066</v>
       </c>
     </row>
-    <row r="245" spans="1:3">
+    <row r="245" hidden="1" spans="1:3">
       <c r="A245" t="s">
         <v>230</v>
       </c>
@@ -25347,7 +25346,7 @@
         <v>329.981179337129</v>
       </c>
     </row>
-    <row r="246" spans="1:3">
+    <row r="246" hidden="1" spans="1:3">
       <c r="A246" t="s">
         <v>77</v>
       </c>
@@ -25358,7 +25357,7 @@
         <v>278.806682833426</v>
       </c>
     </row>
-    <row r="247" spans="1:3">
+    <row r="247" hidden="1" spans="1:3">
       <c r="A247" t="s">
         <v>231</v>
       </c>
@@ -25369,7 +25368,7 @@
         <v>331.678620365446</v>
       </c>
     </row>
-    <row r="248" spans="1:3">
+    <row r="248" hidden="1" spans="1:3">
       <c r="A248" t="s">
         <v>232</v>
       </c>
@@ -25380,7 +25379,7 @@
         <v>327.980854384359</v>
       </c>
     </row>
-    <row r="249" spans="1:3">
+    <row r="249" hidden="1" spans="1:3">
       <c r="A249" t="s">
         <v>350</v>
       </c>
@@ -25391,7 +25390,7 @@
         <v>358.8806749646</v>
       </c>
     </row>
-    <row r="250" spans="1:3">
+    <row r="250" hidden="1" spans="1:3">
       <c r="A250" t="s">
         <v>368</v>
       </c>
@@ -25402,7 +25401,7 @@
         <v>270.319982177734</v>
       </c>
     </row>
-    <row r="251" spans="1:3">
+    <row r="251" hidden="1" spans="1:3">
       <c r="A251" t="s">
         <v>30</v>
       </c>
@@ -25413,7 +25412,7 @@
         <v>285.627911336263</v>
       </c>
     </row>
-    <row r="252" spans="1:3">
+    <row r="252" hidden="1" spans="1:3">
       <c r="A252" t="s">
         <v>233</v>
       </c>
@@ -25424,7 +25423,7 @@
         <v>309.017508738403</v>
       </c>
     </row>
-    <row r="253" spans="1:3">
+    <row r="253" hidden="1" spans="1:3">
       <c r="A253" t="s">
         <v>78</v>
       </c>
@@ -25435,7 +25434,7 @@
         <v>273.423838846232</v>
       </c>
     </row>
-    <row r="254" spans="1:3">
+    <row r="254" hidden="1" spans="1:3">
       <c r="A254" t="s">
         <v>234</v>
       </c>
@@ -25446,7 +25445,7 @@
         <v>314.014530307181</v>
       </c>
     </row>
-    <row r="255" spans="1:3">
+    <row r="255" hidden="1" spans="1:3">
       <c r="A255" t="s">
         <v>235</v>
       </c>
@@ -25457,7 +25456,7 @@
         <v>220.955022655843</v>
       </c>
     </row>
-    <row r="256" spans="1:3">
+    <row r="256" hidden="1" spans="1:3">
       <c r="A256" t="s">
         <v>298</v>
       </c>
@@ -25468,7 +25467,7 @@
         <v>281.923195547485</v>
       </c>
     </row>
-    <row r="257" spans="1:3">
+    <row r="257" hidden="1" spans="1:3">
       <c r="A257" t="s">
         <v>236</v>
       </c>
@@ -25479,7 +25478,7 @@
         <v>287.614758947957</v>
       </c>
     </row>
-    <row r="258" spans="1:3">
+    <row r="258" hidden="1" spans="1:3">
       <c r="A258" t="s">
         <v>355</v>
       </c>
@@ -25490,7 +25489,7 @@
         <v>344.111252502441</v>
       </c>
     </row>
-    <row r="259" spans="1:3">
+    <row r="259" hidden="1" spans="1:3">
       <c r="A259" t="s">
         <v>237</v>
       </c>
@@ -25501,7 +25500,7 @@
         <v>392.086345531936</v>
       </c>
     </row>
-    <row r="260" spans="1:3">
+    <row r="260" hidden="1" spans="1:3">
       <c r="A260" t="s">
         <v>238</v>
       </c>
@@ -25512,7 +25511,7 @@
         <v>272.536322926839</v>
       </c>
     </row>
-    <row r="261" spans="1:3">
+    <row r="261" hidden="1" spans="1:3">
       <c r="A261" t="s">
         <v>239</v>
       </c>
@@ -25523,7 +25522,7 @@
         <v>300.639098574015</v>
       </c>
     </row>
-    <row r="262" spans="1:3">
+    <row r="262" hidden="1" spans="1:3">
       <c r="A262" t="s">
         <v>79</v>
       </c>
@@ -25534,7 +25533,7 @@
         <v>293.30624906311</v>
       </c>
     </row>
-    <row r="263" spans="1:3">
+    <row r="263" hidden="1" spans="1:3">
       <c r="A263" t="s">
         <v>240</v>
       </c>
@@ -25545,7 +25544,7 @@
         <v>443.901131061954</v>
       </c>
     </row>
-    <row r="264" spans="1:3">
+    <row r="264" hidden="1" spans="1:3">
       <c r="A264" t="s">
         <v>241</v>
       </c>
@@ -25556,7 +25555,7 @@
         <v>218.858485547166</v>
       </c>
     </row>
-    <row r="265" spans="1:3">
+    <row r="265" hidden="1" spans="1:3">
       <c r="A265" t="s">
         <v>242</v>
       </c>
@@ -25567,7 +25566,7 @@
         <v>331.783051595052</v>
       </c>
     </row>
-    <row r="266" spans="1:3">
+    <row r="266" hidden="1" spans="1:3">
       <c r="A266" t="s">
         <v>243</v>
       </c>
@@ -25578,7 +25577,7 @@
         <v>458.820220251465</v>
       </c>
     </row>
-    <row r="267" spans="1:3">
+    <row r="267" hidden="1" spans="1:3">
       <c r="A267" t="s">
         <v>31</v>
       </c>
@@ -25589,7 +25588,7 @@
         <v>279.028359132313</v>
       </c>
     </row>
-    <row r="268" spans="1:3">
+    <row r="268" hidden="1" spans="1:3">
       <c r="A268" t="s">
         <v>244</v>
       </c>
@@ -25600,7 +25599,7 @@
         <v>362.85999684361</v>
       </c>
     </row>
-    <row r="269" spans="1:3">
+    <row r="269" hidden="1" spans="1:3">
       <c r="A269" t="s">
         <v>245</v>
       </c>
@@ -25611,7 +25610,7 @@
         <v>321.727416651611</v>
       </c>
     </row>
-    <row r="270" spans="1:3">
+    <row r="270" hidden="1" spans="1:3">
       <c r="A270" t="s">
         <v>246</v>
       </c>
@@ -25622,7 +25621,7 @@
         <v>374.820454719814</v>
       </c>
     </row>
-    <row r="271" spans="1:3">
+    <row r="271" hidden="1" spans="1:3">
       <c r="A271" t="s">
         <v>247</v>
       </c>
@@ -25633,7 +25632,7 @@
         <v>284.335666342367</v>
       </c>
     </row>
-    <row r="272" spans="1:3">
+    <row r="272" hidden="1" spans="1:3">
       <c r="A272" t="s">
         <v>248</v>
       </c>
@@ -25644,7 +25643,7 @@
         <v>340.810936584473</v>
       </c>
     </row>
-    <row r="273" spans="1:3">
+    <row r="273" hidden="1" spans="1:3">
       <c r="A273" t="s">
         <v>249</v>
       </c>
@@ -25655,7 +25654,7 @@
         <v>228.368745934041</v>
       </c>
     </row>
-    <row r="274" spans="1:3">
+    <row r="274" hidden="1" spans="1:3">
       <c r="A274" t="s">
         <v>32</v>
       </c>
@@ -25666,7 +25665,7 @@
         <v>266.996347805379</v>
       </c>
     </row>
-    <row r="275" spans="1:3">
+    <row r="275" hidden="1" spans="1:3">
       <c r="A275" t="s">
         <v>33</v>
       </c>
@@ -25677,7 +25676,7 @@
         <v>282.314931069946</v>
       </c>
     </row>
-    <row r="276" spans="1:3">
+    <row r="276" hidden="1" spans="1:3">
       <c r="A276" t="s">
         <v>80</v>
       </c>
@@ -25688,7 +25687,7 @@
         <v>313.530671806524</v>
       </c>
     </row>
-    <row r="277" spans="1:3">
+    <row r="277" hidden="1" spans="1:3">
       <c r="A277" t="s">
         <v>81</v>
       </c>
@@ -25699,7 +25698,7 @@
         <v>272.312120328369</v>
       </c>
     </row>
-    <row r="278" spans="1:3">
+    <row r="278" hidden="1" spans="1:3">
       <c r="A278" t="s">
         <v>299</v>
       </c>
@@ -25710,7 +25709,7 @@
         <v>282.673636394198</v>
       </c>
     </row>
-    <row r="279" spans="1:3">
+    <row r="279" hidden="1" spans="1:3">
       <c r="A279" t="s">
         <v>250</v>
       </c>
@@ -25721,7 +25720,7 @@
         <v>263.764207662964</v>
       </c>
     </row>
-    <row r="280" spans="1:3">
+    <row r="280" hidden="1" spans="1:3">
       <c r="A280" t="s">
         <v>251</v>
       </c>
@@ -25743,7 +25742,7 @@
         <v>310.992451258341</v>
       </c>
     </row>
-    <row r="282" spans="1:3">
+    <row r="282" hidden="1" spans="1:3">
       <c r="A282" t="s">
         <v>253</v>
       </c>
@@ -25754,7 +25753,7 @@
         <v>235.891280556234</v>
       </c>
     </row>
-    <row r="283" spans="1:3">
+    <row r="283" hidden="1" spans="1:3">
       <c r="A283" t="s">
         <v>95</v>
       </c>
@@ -25776,7 +25775,7 @@
         <v>319.745094686076</v>
       </c>
     </row>
-    <row r="285" spans="1:3">
+    <row r="285" hidden="1" spans="1:3">
       <c r="A285" t="s">
         <v>254</v>
       </c>
@@ -25787,7 +25786,7 @@
         <v>227.865044002075</v>
       </c>
     </row>
-    <row r="286" spans="1:3">
+    <row r="286" hidden="1" spans="1:3">
       <c r="A286" t="s">
         <v>255</v>
       </c>
@@ -25798,7 +25797,7 @@
         <v>228.713000683594</v>
       </c>
     </row>
-    <row r="287" spans="1:3">
+    <row r="287" hidden="1" spans="1:3">
       <c r="A287" t="s">
         <v>256</v>
       </c>
@@ -25809,7 +25808,7 @@
         <v>433.876583432152</v>
       </c>
     </row>
-    <row r="288" spans="1:3">
+    <row r="288" hidden="1" spans="1:3">
       <c r="A288" t="s">
         <v>257</v>
       </c>
@@ -25820,7 +25819,7 @@
         <v>407.406768884568</v>
       </c>
     </row>
-    <row r="289" spans="1:3">
+    <row r="289" hidden="1" spans="1:3">
       <c r="A289" t="s">
         <v>258</v>
       </c>
@@ -25831,7 +25830,7 @@
         <v>350.655306243897</v>
       </c>
     </row>
-    <row r="290" spans="1:3">
+    <row r="290" hidden="1" spans="1:3">
       <c r="A290" t="s">
         <v>259</v>
       </c>
@@ -25842,7 +25841,7 @@
         <v>374.51460516154</v>
       </c>
     </row>
-    <row r="291" spans="1:3">
+    <row r="291" hidden="1" spans="1:3">
       <c r="A291" t="s">
         <v>34</v>
       </c>
@@ -25853,7 +25852,7 @@
         <v>273.25889553772</v>
       </c>
     </row>
-    <row r="292" spans="1:3">
+    <row r="292" hidden="1" spans="1:3">
       <c r="A292" t="s">
         <v>337</v>
       </c>
@@ -25864,7 +25863,7 @@
         <v>311.573719344451</v>
       </c>
     </row>
-    <row r="293" spans="1:3">
+    <row r="293" hidden="1" spans="1:3">
       <c r="A293" t="s">
         <v>260</v>
       </c>
@@ -25875,7 +25874,7 @@
         <v>225.022076313322</v>
       </c>
     </row>
-    <row r="294" spans="1:3">
+    <row r="294" hidden="1" spans="1:3">
       <c r="A294" t="s">
         <v>338</v>
       </c>
@@ -25886,7 +25885,7 @@
         <v>325.181776407267</v>
       </c>
     </row>
-    <row r="295" spans="1:3">
+    <row r="295" hidden="1" spans="1:3">
       <c r="A295" t="s">
         <v>35</v>
       </c>
@@ -25897,7 +25896,7 @@
         <v>346.784240598551</v>
       </c>
     </row>
-    <row r="296" spans="1:3">
+    <row r="296" hidden="1" spans="1:3">
       <c r="A296" t="s">
         <v>36</v>
       </c>
@@ -25908,7 +25907,7 @@
         <v>249.159436706543</v>
       </c>
     </row>
-    <row r="297" spans="1:3">
+    <row r="297" hidden="1" spans="1:3">
       <c r="A297" t="s">
         <v>82</v>
       </c>
@@ -25919,7 +25918,7 @@
         <v>297.361816127116</v>
       </c>
     </row>
-    <row r="298" spans="1:3">
+    <row r="298" hidden="1" spans="1:3">
       <c r="A298" t="s">
         <v>109</v>
       </c>
@@ -25930,7 +25929,7 @@
         <v>257.874680373128</v>
       </c>
     </row>
-    <row r="299" spans="1:3">
+    <row r="299" hidden="1" spans="1:3">
       <c r="A299" t="s">
         <v>261</v>
       </c>
@@ -25952,7 +25951,7 @@
         <v>274.419409423828</v>
       </c>
     </row>
-    <row r="301" spans="1:3">
+    <row r="301" hidden="1" spans="1:3">
       <c r="A301" t="s">
         <v>37</v>
       </c>
@@ -25963,7 +25962,7 @@
         <v>234.714913963013</v>
       </c>
     </row>
-    <row r="302" spans="1:3">
+    <row r="302" hidden="1" spans="1:3">
       <c r="A302" t="s">
         <v>262</v>
       </c>
@@ -25974,7 +25973,7 @@
         <v>368.232397208077</v>
       </c>
     </row>
-    <row r="303" spans="1:3">
+    <row r="303" hidden="1" spans="1:3">
       <c r="A303" t="s">
         <v>263</v>
       </c>
@@ -25985,7 +25984,7 @@
         <v>415.947517088523</v>
       </c>
     </row>
-    <row r="304" spans="1:3">
+    <row r="304" hidden="1" spans="1:3">
       <c r="A304" t="s">
         <v>264</v>
       </c>
@@ -25996,7 +25995,7 @@
         <v>368.23057641916</v>
       </c>
     </row>
-    <row r="305" spans="1:3">
+    <row r="305" hidden="1" spans="1:3">
       <c r="A305" t="s">
         <v>38</v>
       </c>
@@ -26007,7 +26006,7 @@
         <v>279.028359132313</v>
       </c>
     </row>
-    <row r="306" spans="1:3">
+    <row r="306" hidden="1" spans="1:3">
       <c r="A306" t="s">
         <v>83</v>
       </c>
@@ -26018,7 +26017,7 @@
         <v>266.652883320884</v>
       </c>
     </row>
-    <row r="307" spans="1:3">
+    <row r="307" hidden="1" spans="1:3">
       <c r="A307" t="s">
         <v>39</v>
       </c>
@@ -26029,7 +26028,7 @@
         <v>305.390343276977</v>
       </c>
     </row>
-    <row r="308" spans="1:3">
+    <row r="308" hidden="1" spans="1:3">
       <c r="A308" t="s">
         <v>84</v>
       </c>
@@ -26040,7 +26039,7 @@
         <v>256.671657008435</v>
       </c>
     </row>
-    <row r="309" spans="1:3">
+    <row r="309" hidden="1" spans="1:3">
       <c r="A309" t="s">
         <v>265</v>
       </c>
@@ -26062,7 +26061,7 @@
         <v>305.000461785997</v>
       </c>
     </row>
-    <row r="311" spans="1:3">
+    <row r="311" hidden="1" spans="1:3">
       <c r="A311" t="s">
         <v>341</v>
       </c>
@@ -26073,7 +26072,7 @@
         <v>300.230215197754</v>
       </c>
     </row>
-    <row r="312" spans="1:3">
+    <row r="312" hidden="1" spans="1:3">
       <c r="A312" t="s">
         <v>266</v>
       </c>
@@ -26084,7 +26083,7 @@
         <v>220.467879589698</v>
       </c>
     </row>
-    <row r="313" spans="1:3">
+    <row r="313" hidden="1" spans="1:3">
       <c r="A313" t="s">
         <v>94</v>
       </c>
@@ -26095,7 +26094,7 @@
         <v>293.556306652222</v>
       </c>
     </row>
-    <row r="314" spans="1:3">
+    <row r="314" hidden="1" spans="1:3">
       <c r="A314" t="s">
         <v>267</v>
       </c>
@@ -26106,7 +26105,7 @@
         <v>229.620712825811</v>
       </c>
     </row>
-    <row r="315" spans="1:3">
+    <row r="315" hidden="1" spans="1:3">
       <c r="A315" t="s">
         <v>268</v>
       </c>
@@ -26117,7 +26116,7 @@
         <v>353.723749006871</v>
       </c>
     </row>
-    <row r="316" spans="1:3">
+    <row r="316" hidden="1" spans="1:3">
       <c r="A316" t="s">
         <v>269</v>
       </c>
@@ -26128,7 +26127,7 @@
         <v>297.912022397577</v>
       </c>
     </row>
-    <row r="317" spans="1:3">
+    <row r="317" hidden="1" spans="1:3">
       <c r="A317" t="s">
         <v>342</v>
       </c>
@@ -26139,7 +26138,7 @@
         <v>295.586242248535</v>
       </c>
     </row>
-    <row r="318" spans="1:3">
+    <row r="318" hidden="1" spans="1:3">
       <c r="A318" t="s">
         <v>270</v>
       </c>
@@ -26150,7 +26149,7 @@
         <v>289.652510169254</v>
       </c>
     </row>
-    <row r="319" spans="1:3">
+    <row r="319" hidden="1" spans="1:3">
       <c r="A319" t="s">
         <v>85</v>
       </c>
@@ -26161,7 +26160,7 @@
         <v>278.806682833426</v>
       </c>
     </row>
-    <row r="320" spans="1:3">
+    <row r="320" hidden="1" spans="1:3">
       <c r="A320" t="s">
         <v>40</v>
       </c>
@@ -26172,7 +26171,7 @@
         <v>276.431482975842</v>
       </c>
     </row>
-    <row r="321" spans="1:3">
+    <row r="321" hidden="1" spans="1:3">
       <c r="A321" t="s">
         <v>271</v>
       </c>
@@ -26183,7 +26182,7 @@
         <v>261.282990483805</v>
       </c>
     </row>
-    <row r="322" spans="1:3">
+    <row r="322" hidden="1" spans="1:3">
       <c r="A322" t="s">
         <v>41</v>
       </c>
@@ -26194,7 +26193,7 @@
         <v>296.951784927368</v>
       </c>
     </row>
-    <row r="323" spans="1:3">
+    <row r="323" hidden="1" spans="1:3">
       <c r="A323" t="s">
         <v>343</v>
       </c>
@@ -26205,7 +26204,7 @@
         <v>308.968406191823</v>
       </c>
     </row>
-    <row r="324" spans="1:3">
+    <row r="324" hidden="1" spans="1:3">
       <c r="A324" t="s">
         <v>300</v>
       </c>
@@ -26216,7 +26215,7 @@
         <v>308.348718811035</v>
       </c>
     </row>
-    <row r="325" spans="1:3">
+    <row r="325" hidden="1" spans="1:3">
       <c r="A325" t="s">
         <v>86</v>
       </c>
@@ -26227,7 +26226,7 @@
         <v>276.672427334362</v>
       </c>
     </row>
-    <row r="326" spans="1:3">
+    <row r="326" hidden="1" spans="1:3">
       <c r="A326" t="s">
         <v>309</v>
       </c>
@@ -26238,7 +26237,7 @@
         <v>251.395597635178</v>
       </c>
     </row>
-    <row r="327" spans="1:3">
+    <row r="327" hidden="1" spans="1:3">
       <c r="A327" t="s">
         <v>272</v>
       </c>
@@ -26249,7 +26248,7 @@
         <v>298.952033982137</v>
       </c>
     </row>
-    <row r="328" spans="1:3">
+    <row r="328" hidden="1" spans="1:3">
       <c r="A328" t="s">
         <v>369</v>
       </c>
@@ -26271,7 +26270,7 @@
         <v>276.960908025106</v>
       </c>
     </row>
-    <row r="330" spans="1:3">
+    <row r="330" hidden="1" spans="1:3">
       <c r="A330" t="s">
         <v>87</v>
       </c>
@@ -26282,7 +26281,7 @@
         <v>260.751515623576</v>
       </c>
     </row>
-    <row r="331" spans="1:3">
+    <row r="331" hidden="1" spans="1:3">
       <c r="A331" t="s">
         <v>273</v>
       </c>
@@ -26293,7 +26292,7 @@
         <v>339.200232055257</v>
       </c>
     </row>
-    <row r="332" spans="1:3">
+    <row r="332" hidden="1" spans="1:3">
       <c r="A332" t="s">
         <v>274</v>
       </c>
@@ -26304,7 +26303,7 @@
         <v>193.932482492269</v>
       </c>
     </row>
-    <row r="333" spans="1:3">
+    <row r="333" hidden="1" spans="1:3">
       <c r="A333" t="s">
         <v>275</v>
       </c>
@@ -26315,7 +26314,7 @@
         <v>241.634852592773</v>
       </c>
     </row>
-    <row r="334" spans="1:3">
+    <row r="334" hidden="1" spans="1:3">
       <c r="A334" t="s">
         <v>345</v>
       </c>
@@ -26326,7 +26325,7 @@
         <v>301.176327819824</v>
       </c>
     </row>
-    <row r="335" spans="1:3">
+    <row r="335" hidden="1" spans="1:3">
       <c r="A335" t="s">
         <v>276</v>
       </c>
@@ -26337,7 +26336,7 @@
         <v>402.544213970657</v>
       </c>
     </row>
-    <row r="336" spans="1:3">
+    <row r="336" hidden="1" spans="1:3">
       <c r="A336" t="s">
         <v>42</v>
       </c>
@@ -26348,7 +26347,7 @@
         <v>273.974973236084</v>
       </c>
     </row>
-    <row r="337" spans="1:3">
+    <row r="337" hidden="1" spans="1:3">
       <c r="A337" t="s">
         <v>370</v>
       </c>
@@ -26359,7 +26358,7 @@
         <v>294.217692001343</v>
       </c>
     </row>
-    <row r="338" spans="1:3">
+    <row r="338" hidden="1" spans="1:3">
       <c r="A338" t="s">
         <v>88</v>
       </c>
@@ -26370,7 +26369,7 @@
         <v>249.976689334107</v>
       </c>
     </row>
-    <row r="339" spans="1:3">
+    <row r="339" hidden="1" spans="1:3">
       <c r="A339" t="s">
         <v>277</v>
       </c>
@@ -26381,7 +26380,7 @@
         <v>322.081999744738</v>
       </c>
     </row>
-    <row r="340" spans="1:3">
+    <row r="340" hidden="1" spans="1:3">
       <c r="A340" t="s">
         <v>278</v>
       </c>
@@ -26414,7 +26413,7 @@
         <v>325.278744584147</v>
       </c>
     </row>
-    <row r="343" spans="1:3">
+    <row r="343" hidden="1" spans="1:3">
       <c r="A343" t="s">
         <v>89</v>
       </c>
@@ -26425,7 +26424,7 @@
         <v>266.766198355103</v>
       </c>
     </row>
-    <row r="344" spans="1:3">
+    <row r="344" hidden="1" spans="1:3">
       <c r="A344" t="s">
         <v>280</v>
       </c>
@@ -26436,7 +26435,7 @@
         <v>302.412601607259</v>
       </c>
     </row>
-    <row r="345" spans="1:3">
+    <row r="345" hidden="1" spans="1:3">
       <c r="A345" t="s">
         <v>281</v>
       </c>
@@ -26447,7 +26446,7 @@
         <v>218.858485547166</v>
       </c>
     </row>
-    <row r="346" spans="1:3">
+    <row r="346" hidden="1" spans="1:3">
       <c r="A346" t="s">
         <v>282</v>
       </c>
@@ -26458,7 +26457,7 @@
         <v>286.925357948405</v>
       </c>
     </row>
-    <row r="347" spans="1:3">
+    <row r="347" hidden="1" spans="1:3">
       <c r="A347" t="s">
         <v>283</v>
       </c>
@@ -26469,7 +26468,7 @@
         <v>371.895806586507</v>
       </c>
     </row>
-    <row r="348" spans="1:3">
+    <row r="348" hidden="1" spans="1:3">
       <c r="A348" t="s">
         <v>284</v>
       </c>
@@ -26480,7 +26479,7 @@
         <v>265.214281174723</v>
       </c>
     </row>
-    <row r="349" spans="1:3">
+    <row r="349" hidden="1" spans="1:3">
       <c r="A349" t="s">
         <v>285</v>
       </c>
@@ -26491,7 +26490,7 @@
         <v>326.792794545695</v>
       </c>
     </row>
-    <row r="350" spans="1:3">
+    <row r="350" hidden="1" spans="1:3">
       <c r="A350" t="s">
         <v>346</v>
       </c>
@@ -26502,7 +26501,7 @@
         <v>288.618571827799</v>
       </c>
     </row>
-    <row r="351" spans="1:3">
+    <row r="351" hidden="1" spans="1:3">
       <c r="A351" t="s">
         <v>371</v>
       </c>
@@ -26513,7 +26512,7 @@
         <v>288.13721884257</v>
       </c>
     </row>
-    <row r="352" spans="1:3">
+    <row r="352" hidden="1" spans="1:3">
       <c r="A352" t="s">
         <v>286</v>
       </c>
@@ -26535,7 +26534,7 @@
         <v>335.88718090457</v>
       </c>
     </row>
-    <row r="354" spans="1:3">
+    <row r="354" hidden="1" spans="1:3">
       <c r="A354" t="s">
         <v>287</v>
       </c>
@@ -26546,7 +26545,7 @@
         <v>407.406768884568</v>
       </c>
     </row>
-    <row r="355" spans="1:3">
+    <row r="355" hidden="1" spans="1:3">
       <c r="A355" t="s">
         <v>301</v>
       </c>
@@ -26557,7 +26556,7 @@
         <v>324.077696029663</v>
       </c>
     </row>
-    <row r="356" spans="1:3">
+    <row r="356" hidden="1" spans="1:3">
       <c r="A356" t="s">
         <v>43</v>
       </c>
@@ -26568,7 +26567,7 @@
         <v>279.925999350993</v>
       </c>
     </row>
-    <row r="357" spans="1:3">
+    <row r="357" hidden="1" spans="1:3">
       <c r="A357" t="s">
         <v>288</v>
       </c>
@@ -26590,7 +26589,7 @@
         <v>274.621090271199</v>
       </c>
     </row>
-    <row r="359" spans="1:3">
+    <row r="359" hidden="1" spans="1:3">
       <c r="A359" t="s">
         <v>44</v>
       </c>
@@ -26601,7 +26600,7 @@
         <v>272.016418365479</v>
       </c>
     </row>
-    <row r="360" spans="1:3">
+    <row r="360" hidden="1" spans="1:3">
       <c r="A360" t="s">
         <v>302</v>
       </c>
@@ -26612,7 +26611,7 @@
         <v>339.318702056885</v>
       </c>
     </row>
-    <row r="361" spans="1:3">
+    <row r="361" hidden="1" spans="1:3">
       <c r="A361" t="s">
         <v>289</v>
       </c>
@@ -26623,7 +26622,7 @@
         <v>397.924830148185</v>
       </c>
     </row>
-    <row r="362" spans="1:3">
+    <row r="362" hidden="1" spans="1:3">
       <c r="A362" t="s">
         <v>347</v>
       </c>
@@ -26634,7 +26633,7 @@
         <v>311.573719344451</v>
       </c>
     </row>
-    <row r="363" spans="1:3">
+    <row r="363" hidden="1" spans="1:3">
       <c r="A363" t="s">
         <v>310</v>
       </c>
@@ -26645,7 +26644,7 @@
         <v>251.395597635178</v>
       </c>
     </row>
-    <row r="364" spans="1:3">
+    <row r="364" hidden="1" spans="1:3">
       <c r="A364" t="s">
         <v>290</v>
       </c>
@@ -26656,7 +26655,7 @@
         <v>254.485424772135</v>
       </c>
     </row>
-    <row r="365" spans="1:3">
+    <row r="365" hidden="1" spans="1:3">
       <c r="A365" t="s">
         <v>291</v>
       </c>
@@ -26667,7 +26666,7 @@
         <v>301.084888990682</v>
       </c>
     </row>
-    <row r="366" spans="1:3">
+    <row r="366" hidden="1" spans="1:3">
       <c r="A366" t="s">
         <v>292</v>
       </c>
@@ -26678,7 +26677,7 @@
         <v>260.101962633405</v>
       </c>
     </row>
-    <row r="367" spans="1:3">
+    <row r="367" hidden="1" spans="1:3">
       <c r="A367" t="s">
         <v>293</v>
       </c>
@@ -26689,7 +26688,7 @@
         <v>265.247427846273</v>
       </c>
     </row>
-    <row r="368" spans="1:3">
+    <row r="368" hidden="1" spans="1:3">
       <c r="A368" t="s">
         <v>294</v>
       </c>
@@ -26700,7 +26699,7 @@
         <v>224.65941641866</v>
       </c>
     </row>
-    <row r="369" spans="1:3">
+    <row r="369" hidden="1" spans="1:3">
       <c r="A369" t="s">
         <v>295</v>
       </c>
@@ -26711,7 +26710,7 @@
         <v>240.285245385742</v>
       </c>
     </row>
-    <row r="370" spans="1:3">
+    <row r="370" hidden="1" spans="1:3">
       <c r="A370" t="s">
         <v>372</v>
       </c>
@@ -26722,7 +26721,7 @@
         <v>229.346788659871</v>
       </c>
     </row>
-    <row r="371" spans="1:3">
+    <row r="371" hidden="1" spans="1:3">
       <c r="A371" t="s">
         <v>96</v>
       </c>
@@ -26734,6 +26733,14 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="B1:B371" etc:filterBottomFollowUsedRange="0">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="7"/>
+      </filters>
+    </filterColumn>
+    <extLst/>
+  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>

</xml_diff>